<commit_message>
Add week of 6 Jul 2026 menu, vet, and recipes
- Lock in week of 6 Jul 2026 menu + T1 vet (applies standing prefs:
  no raw veg, less garlic, easy on herbs, more tomato)
- Potato/bread themed: prata Wed, bread days Mon & Fri, potato most days
- Add 8 recipes: pasta arrabbiata, padang chicken curry, tortilla de patatas,
  slow cooker BBQ pulled pork, braised pork tofu & egg (tau yu bak),
  tomato soup, grilled cheese + sheet-tray tomato soup, cubano
- Update dish-rotation cook log + master; kitchen-inventory new items (Out)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -2327,115 +2327,307 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n"/>
+      <c r="A96" s="2" t="n">
+        <v>46208</v>
+      </c>
       <c r="B96" s="3">
         <f>IF(A96="","",TEXT(A96,"ddd"))</f>
         <v/>
       </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Pasta arrabbiata</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n"/>
+      <c r="A97" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="B97" s="3">
         <f>IF(A97="","",TEXT(A97,"ddd"))</f>
         <v/>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Pulled pork burger</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n"/>
+      <c r="A98" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="B98" s="3">
         <f>IF(A98="","",TEXT(A98,"ddd"))</f>
         <v/>
       </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Spanish omelette</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n"/>
+      <c r="A99" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="B99" s="3">
         <f>IF(A99="","",TEXT(A99,"ddd"))</f>
         <v/>
       </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Watercress pork rib soup</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n"/>
+      <c r="A100" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="B100" s="3">
         <f>IF(A100="","",TEXT(A100,"ddd"))</f>
         <v/>
       </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Braised pork with tofu and egg (Tau Yu Bak)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n"/>
+      <c r="A101" s="2" t="n">
+        <v>46210</v>
+      </c>
       <c r="B101" s="3">
         <f>IF(A101="","",TEXT(A101,"ddd"))</f>
         <v/>
       </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Steamed pomfret</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n"/>
+      <c r="A102" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="B102" s="3">
         <f>IF(A102="","",TEXT(A102,"ddd"))</f>
         <v/>
       </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Frozen prata</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n"/>
+      <c r="A103" s="2" t="n">
+        <v>46211</v>
+      </c>
       <c r="B103" s="3">
         <f>IF(A103="","",TEXT(A103,"ddd"))</f>
         <v/>
       </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Padang chicken curry</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n"/>
+      <c r="A104" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="B104" s="3">
         <f>IF(A104="","",TEXT(A104,"ddd"))</f>
         <v/>
       </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Nasi lemak</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n"/>
+      <c r="A105" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="B105" s="3">
         <f>IF(A105="","",TEXT(A105,"ddd"))</f>
         <v/>
       </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Fried chicken wings</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n"/>
+      <c r="A106" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="B106" s="3">
         <f>IF(A106="","",TEXT(A106,"ddd"))</f>
         <v/>
       </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Egg omelette</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n"/>
+      <c r="A107" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="B107" s="3">
         <f>IF(A107="","",TEXT(A107,"ddd"))</f>
         <v/>
       </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Sambal long beans</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026) — sambal kangkong recipe w/ long beans</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n"/>
+      <c r="A108" s="2" t="n">
+        <v>46212</v>
+      </c>
       <c r="B108" s="3">
         <f>IF(A108="","",TEXT(A108,"ddd"))</f>
         <v/>
       </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Begedil</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n"/>
+      <c r="A109" s="2" t="n">
+        <v>46213</v>
+      </c>
       <c r="B109" s="3">
         <f>IF(A109="","",TEXT(A109,"ddd"))</f>
         <v/>
       </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Grilled cheese</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n"/>
+      <c r="A110" s="2" t="n">
+        <v>46213</v>
+      </c>
       <c r="B110" s="3">
         <f>IF(A110="","",TEXT(A110,"ddd"))</f>
         <v/>
       </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Tomato soup</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n"/>
+      <c r="A111" s="2" t="n">
+        <v>46213</v>
+      </c>
       <c r="B111" s="3">
         <f>IF(A111="","",TEXT(A111,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Fries</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>planned (week of 6 Jul 2026)</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -3778,7 +3970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H128"/>
+  <dimension ref="A1:H140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7687,6 +7879,378 @@
       </c>
       <c r="G128">
         <f>IF(C128="","Never cooked",IF(D128&lt;F128,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Pasta arrabbiata</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C129">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A129)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A129)),"")</f>
+        <v/>
+      </c>
+      <c r="D129">
+        <f>IF(C129="","",TODAY()-C129)</f>
+        <v/>
+      </c>
+      <c r="E129">
+        <f>COUNTIF('Cook log'!C2:C1000,A129)</f>
+        <v/>
+      </c>
+      <c r="F129" t="n">
+        <v>21</v>
+      </c>
+      <c r="G129">
+        <f>IF(C129="","Never cooked",IF(D129&lt;F129,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Pulled pork burger</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="C130">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A130)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A130)),"")</f>
+        <v/>
+      </c>
+      <c r="D130">
+        <f>IF(C130="","",TODAY()-C130)</f>
+        <v/>
+      </c>
+      <c r="E130">
+        <f>COUNTIF('Cook log'!C2:C1000,A130)</f>
+        <v/>
+      </c>
+      <c r="F130" t="n">
+        <v>21</v>
+      </c>
+      <c r="G130">
+        <f>IF(C130="","Never cooked",IF(D130&lt;F130,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Spanish omelette</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Egg</t>
+        </is>
+      </c>
+      <c r="C131">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A131)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A131)),"")</f>
+        <v/>
+      </c>
+      <c r="D131">
+        <f>IF(C131="","",TODAY()-C131)</f>
+        <v/>
+      </c>
+      <c r="E131">
+        <f>COUNTIF('Cook log'!C2:C1000,A131)</f>
+        <v/>
+      </c>
+      <c r="F131" t="n">
+        <v>21</v>
+      </c>
+      <c r="G131">
+        <f>IF(C131="","Never cooked",IF(D131&lt;F131,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Luncheon meat &amp; potatoes</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="C132">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A132)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A132)),"")</f>
+        <v/>
+      </c>
+      <c r="D132">
+        <f>IF(C132="","",TODAY()-C132)</f>
+        <v/>
+      </c>
+      <c r="E132">
+        <f>COUNTIF('Cook log'!C2:C1000,A132)</f>
+        <v/>
+      </c>
+      <c r="F132" t="n">
+        <v>21</v>
+      </c>
+      <c r="G132">
+        <f>IF(C132="","Never cooked",IF(D132&lt;F132,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Frozen prata</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C133">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A133)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A133)),"")</f>
+        <v/>
+      </c>
+      <c r="D133">
+        <f>IF(C133="","",TODAY()-C133)</f>
+        <v/>
+      </c>
+      <c r="E133">
+        <f>COUNTIF('Cook log'!C2:C1000,A133)</f>
+        <v/>
+      </c>
+      <c r="F133" t="n">
+        <v>21</v>
+      </c>
+      <c r="G133">
+        <f>IF(C133="","Never cooked",IF(D133&lt;F133,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Padang chicken curry</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="C134">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A134)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A134)),"")</f>
+        <v/>
+      </c>
+      <c r="D134">
+        <f>IF(C134="","",TODAY()-C134)</f>
+        <v/>
+      </c>
+      <c r="E134">
+        <f>COUNTIF('Cook log'!C2:C1000,A134)</f>
+        <v/>
+      </c>
+      <c r="F134" t="n">
+        <v>21</v>
+      </c>
+      <c r="G134">
+        <f>IF(C134="","Never cooked",IF(D134&lt;F134,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Sambal long beans</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C135">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A135)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A135)),"")</f>
+        <v/>
+      </c>
+      <c r="D135">
+        <f>IF(C135="","",TODAY()-C135)</f>
+        <v/>
+      </c>
+      <c r="E135">
+        <f>COUNTIF('Cook log'!C2:C1000,A135)</f>
+        <v/>
+      </c>
+      <c r="F135" t="n">
+        <v>21</v>
+      </c>
+      <c r="G135">
+        <f>IF(C135="","Never cooked",IF(D135&lt;F135,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Begedil</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C136">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A136)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A136)),"")</f>
+        <v/>
+      </c>
+      <c r="D136">
+        <f>IF(C136="","",TODAY()-C136)</f>
+        <v/>
+      </c>
+      <c r="E136">
+        <f>COUNTIF('Cook log'!C2:C1000,A136)</f>
+        <v/>
+      </c>
+      <c r="F136" t="n">
+        <v>21</v>
+      </c>
+      <c r="G136">
+        <f>IF(C136="","Never cooked",IF(D136&lt;F136,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Grilled cheese</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C137">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A137)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A137)),"")</f>
+        <v/>
+      </c>
+      <c r="D137">
+        <f>IF(C137="","",TODAY()-C137)</f>
+        <v/>
+      </c>
+      <c r="E137">
+        <f>COUNTIF('Cook log'!C2:C1000,A137)</f>
+        <v/>
+      </c>
+      <c r="F137" t="n">
+        <v>21</v>
+      </c>
+      <c r="G137">
+        <f>IF(C137="","Never cooked",IF(D137&lt;F137,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Tomato soup</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="C138">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A138)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A138)),"")</f>
+        <v/>
+      </c>
+      <c r="D138">
+        <f>IF(C138="","",TODAY()-C138)</f>
+        <v/>
+      </c>
+      <c r="E138">
+        <f>COUNTIF('Cook log'!C2:C1000,A138)</f>
+        <v/>
+      </c>
+      <c r="F138" t="n">
+        <v>21</v>
+      </c>
+      <c r="G138">
+        <f>IF(C138="","Never cooked",IF(D138&lt;F138,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Fries</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C139">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A139)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A139)),"")</f>
+        <v/>
+      </c>
+      <c r="D139">
+        <f>IF(C139="","",TODAY()-C139)</f>
+        <v/>
+      </c>
+      <c r="E139">
+        <f>COUNTIF('Cook log'!C2:C1000,A139)</f>
+        <v/>
+      </c>
+      <c r="F139" t="n">
+        <v>21</v>
+      </c>
+      <c r="G139">
+        <f>IF(C139="","Never cooked",IF(D139&lt;F139,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Braised pork with tofu and egg (Tau Yu Bak)</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="C140">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A140)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A140)),"")</f>
+        <v/>
+      </c>
+      <c r="D140">
+        <f>IF(C140="","",TODAY()-C140)</f>
+        <v/>
+      </c>
+      <c r="E140">
+        <f>COUNTIF('Cook log'!C2:C1000,A140)</f>
+        <v/>
+      </c>
+      <c r="F140" t="n">
+        <v>21</v>
+      </c>
+      <c r="G140">
+        <f>IF(C140="","Never cooked",IF(D140&lt;F140,"Cooldown","Due"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add weeks of 13 Jul & 20 Jul 2026 menus, vets, and recipes
- Week of 13 Jul (local/comfort: dry laksa, hamburg, Portuguese chicken
  rice, chicken curry + roti, baby back ribs) + T1 vet
- Week of 20 Jul (gentle home-style, no tomato/seafood/sesame/strong smells:
  sticky pork belly, teriyaki, hokkien hai fan, pork rib king, fried beehoon)
  + T1 vet
- Add recipes: japanese hamburg patty, macau portuguese chicken rice,
  dry mee siam, chicken curry with potato, baby back ribs, chicken parm
  sandwich, meatball marinara sub
- Update dish-rotation cook log + master; kitchen-inventory new items (Out)
- Memory: recorded T1 nausea aversions (no sesame oil, avoid seafood,
  avoid strong-smelling dishes, tomato now variable)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -2631,171 +2631,459 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n"/>
+      <c r="A112" s="2" t="n">
+        <v>46216</v>
+      </c>
       <c r="B112" s="3">
         <f>IF(A112="","",TEXT(A112,"ddd"))</f>
         <v/>
       </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Dry laksa</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n"/>
+      <c r="A113" s="2" t="n">
+        <v>46216</v>
+      </c>
       <c r="B113" s="3">
         <f>IF(A113="","",TEXT(A113,"ddd"))</f>
         <v/>
       </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Fishball minced pork soup</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n"/>
+      <c r="A114" s="2" t="n">
+        <v>46217</v>
+      </c>
       <c r="B114" s="3">
         <f>IF(A114="","",TEXT(A114,"ddd"))</f>
         <v/>
       </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Japanese hamburg patty</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n"/>
+      <c r="A115" s="2" t="n">
+        <v>46217</v>
+      </c>
       <c r="B115" s="3">
         <f>IF(A115="","",TEXT(A115,"ddd"))</f>
         <v/>
       </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n"/>
+      <c r="A116" s="2" t="n">
+        <v>46217</v>
+      </c>
       <c r="B116" s="3">
         <f>IF(A116="","",TEXT(A116,"ddd"))</f>
         <v/>
       </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Stir fried dou miao</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n"/>
+      <c r="A117" s="2" t="n">
+        <v>46218</v>
+      </c>
       <c r="B117" s="3">
         <f>IF(A117="","",TEXT(A117,"ddd"))</f>
         <v/>
       </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Macau Portuguese chicken rice</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n"/>
+      <c r="A118" s="2" t="n">
+        <v>46218</v>
+      </c>
       <c r="B118" s="3">
         <f>IF(A118="","",TEXT(A118,"ddd"))</f>
         <v/>
       </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ABC soup</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n"/>
+      <c r="A119" s="2" t="n">
+        <v>46219</v>
+      </c>
       <c r="B119" s="3">
         <f>IF(A119="","",TEXT(A119,"ddd"))</f>
         <v/>
       </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Bread</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026) — with curry</t>
+        </is>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n"/>
+      <c r="A120" s="2" t="n">
+        <v>46219</v>
+      </c>
       <c r="B120" s="3">
         <f>IF(A120="","",TEXT(A120,"ddd"))</f>
         <v/>
       </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Chicken curry</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n"/>
+      <c r="A121" s="2" t="n">
+        <v>46220</v>
+      </c>
       <c r="B121" s="3">
         <f>IF(A121="","",TEXT(A121,"ddd"))</f>
         <v/>
       </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Baby back ribs</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n"/>
+      <c r="A122" s="2" t="n">
+        <v>46220</v>
+      </c>
       <c r="B122" s="3">
         <f>IF(A122="","",TEXT(A122,"ddd"))</f>
         <v/>
       </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Cornbread</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n"/>
+      <c r="A123" s="2" t="n">
+        <v>46220</v>
+      </c>
       <c r="B123" s="3">
         <f>IF(A123="","",TEXT(A123,"ddd"))</f>
         <v/>
       </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Creamed spinach</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>planned (week of 13 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n"/>
+      <c r="A124" s="2" t="n">
+        <v>46223</v>
+      </c>
       <c r="B124" s="3">
         <f>IF(A124="","",TEXT(A124,"ddd"))</f>
         <v/>
       </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sticky pork belly</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n"/>
+      <c r="A125" s="2" t="n">
+        <v>46223</v>
+      </c>
       <c r="B125" s="3">
         <f>IF(A125="","",TEXT(A125,"ddd"))</f>
         <v/>
       </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n"/>
+      <c r="A126" s="2" t="n">
+        <v>46223</v>
+      </c>
       <c r="B126" s="3">
         <f>IF(A126="","",TEXT(A126,"ddd"))</f>
         <v/>
       </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Winter melon pork rib soup</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n"/>
+      <c r="A127" s="2" t="n">
+        <v>46224</v>
+      </c>
       <c r="B127" s="3">
         <f>IF(A127="","",TEXT(A127,"ddd"))</f>
         <v/>
       </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Teriyaki chicken cutlet</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n"/>
+      <c r="A128" s="2" t="n">
+        <v>46224</v>
+      </c>
       <c r="B128" s="3">
         <f>IF(A128="","",TEXT(A128,"ddd"))</f>
         <v/>
       </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Rösti</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n"/>
+      <c r="A129" s="2" t="n">
+        <v>46224</v>
+      </c>
       <c r="B129" s="3">
         <f>IF(A129="","",TEXT(A129,"ddd"))</f>
         <v/>
       </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Broccoli stir fry with mushroom</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n"/>
+      <c r="A130" s="2" t="n">
+        <v>46225</v>
+      </c>
       <c r="B130" s="3">
         <f>IF(A130="","",TEXT(A130,"ddd"))</f>
         <v/>
       </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Hokkien hai fan (ah gong)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n"/>
+      <c r="A131" s="2" t="n">
+        <v>46226</v>
+      </c>
       <c r="B131" s="3">
         <f>IF(A131="","",TEXT(A131,"ddd"))</f>
         <v/>
       </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Pork rib king</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n"/>
+      <c r="A132" s="2" t="n">
+        <v>46226</v>
+      </c>
       <c r="B132" s="3">
         <f>IF(A132="","",TEXT(A132,"ddd"))</f>
         <v/>
       </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Steamed egg (ah gong style)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n"/>
+      <c r="A133" s="2" t="n">
+        <v>46226</v>
+      </c>
       <c r="B133" s="3">
         <f>IF(A133="","",TEXT(A133,"ddd"))</f>
         <v/>
       </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Stir-fried baby bok choy</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n"/>
+      <c r="A134" s="2" t="n">
+        <v>46227</v>
+      </c>
       <c r="B134" s="3">
         <f>IF(A134="","",TEXT(A134,"ddd"))</f>
         <v/>
       </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Stir fried bee hoon</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026) — no prawns</t>
+        </is>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n"/>
+      <c r="A135" s="2" t="n">
+        <v>46227</v>
+      </c>
       <c r="B135" s="3">
         <f>IF(A135="","",TEXT(A135,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Fried chicken wings</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>planned (week of 20 Jul 2026)</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -3970,7 +4258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8251,6 +8539,347 @@
       </c>
       <c r="G140">
         <f>IF(C140="","Never cooked",IF(D140&lt;F140,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Dry laksa</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C141">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A141)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A141)),"")</f>
+        <v/>
+      </c>
+      <c r="D141">
+        <f>IF(C141="","",TODAY()-C141)</f>
+        <v/>
+      </c>
+      <c r="E141">
+        <f>COUNTIF('Cook log'!C2:C1000,A141)</f>
+        <v/>
+      </c>
+      <c r="F141" t="n">
+        <v>21</v>
+      </c>
+      <c r="G141">
+        <f>IF(C141="","Never cooked",IF(D141&lt;F141,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Japanese hamburg patty</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Beef</t>
+        </is>
+      </c>
+      <c r="C142">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A142)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A142)),"")</f>
+        <v/>
+      </c>
+      <c r="D142">
+        <f>IF(C142="","",TODAY()-C142)</f>
+        <v/>
+      </c>
+      <c r="E142">
+        <f>COUNTIF('Cook log'!C2:C1000,A142)</f>
+        <v/>
+      </c>
+      <c r="F142" t="n">
+        <v>21</v>
+      </c>
+      <c r="G142">
+        <f>IF(C142="","Never cooked",IF(D142&lt;F142,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Dry mee siam</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Noodle</t>
+        </is>
+      </c>
+      <c r="C143">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A143)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A143)),"")</f>
+        <v/>
+      </c>
+      <c r="D143">
+        <f>IF(C143="","",TODAY()-C143)</f>
+        <v/>
+      </c>
+      <c r="E143">
+        <f>COUNTIF('Cook log'!C2:C1000,A143)</f>
+        <v/>
+      </c>
+      <c r="F143" t="n">
+        <v>21</v>
+      </c>
+      <c r="G143">
+        <f>IF(C143="","Never cooked",IF(D143&lt;F143,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Chicken curry</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="C144">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A144)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A144)),"")</f>
+        <v/>
+      </c>
+      <c r="D144">
+        <f>IF(C144="","",TODAY()-C144)</f>
+        <v/>
+      </c>
+      <c r="E144">
+        <f>COUNTIF('Cook log'!C2:C1000,A144)</f>
+        <v/>
+      </c>
+      <c r="F144" t="n">
+        <v>21</v>
+      </c>
+      <c r="G144">
+        <f>IF(C144="","Never cooked",IF(D144&lt;F144,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Baby back ribs</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="C145">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A145)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A145)),"")</f>
+        <v/>
+      </c>
+      <c r="D145">
+        <f>IF(C145="","",TODAY()-C145)</f>
+        <v/>
+      </c>
+      <c r="E145">
+        <f>COUNTIF('Cook log'!C2:C1000,A145)</f>
+        <v/>
+      </c>
+      <c r="F145" t="n">
+        <v>21</v>
+      </c>
+      <c r="G145">
+        <f>IF(C145="","Never cooked",IF(D145&lt;F145,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Cornbread</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C146">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A146)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A146)),"")</f>
+        <v/>
+      </c>
+      <c r="D146">
+        <f>IF(C146="","",TODAY()-C146)</f>
+        <v/>
+      </c>
+      <c r="E146">
+        <f>COUNTIF('Cook log'!C2:C1000,A146)</f>
+        <v/>
+      </c>
+      <c r="F146" t="n">
+        <v>21</v>
+      </c>
+      <c r="G146">
+        <f>IF(C146="","Never cooked",IF(D146&lt;F146,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Creamed spinach</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C147">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A147)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A147)),"")</f>
+        <v/>
+      </c>
+      <c r="D147">
+        <f>IF(C147="","",TODAY()-C147)</f>
+        <v/>
+      </c>
+      <c r="E147">
+        <f>COUNTIF('Cook log'!C2:C1000,A147)</f>
+        <v/>
+      </c>
+      <c r="F147" t="n">
+        <v>21</v>
+      </c>
+      <c r="G147">
+        <f>IF(C147="","Never cooked",IF(D147&lt;F147,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C148">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A148)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A148)),"")</f>
+        <v/>
+      </c>
+      <c r="D148">
+        <f>IF(C148="","",TODAY()-C148)</f>
+        <v/>
+      </c>
+      <c r="E148">
+        <f>COUNTIF('Cook log'!C2:C1000,A148)</f>
+        <v/>
+      </c>
+      <c r="F148" t="n">
+        <v>14</v>
+      </c>
+      <c r="G148">
+        <f>IF(C148="","Never cooked",IF(D148&lt;F148,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Bread</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C149">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A149)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A149)),"")</f>
+        <v/>
+      </c>
+      <c r="D149">
+        <f>IF(C149="","",TODAY()-C149)</f>
+        <v/>
+      </c>
+      <c r="E149">
+        <f>COUNTIF('Cook log'!C2:C1000,A149)</f>
+        <v/>
+      </c>
+      <c r="F149" t="n">
+        <v>14</v>
+      </c>
+      <c r="G149">
+        <f>IF(C149="","Never cooked",IF(D149&lt;F149,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Hokkien hai fan (ah gong)</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C150">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A150)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A150)),"")</f>
+        <v/>
+      </c>
+      <c r="D150">
+        <f>IF(C150="","",TODAY()-C150)</f>
+        <v/>
+      </c>
+      <c r="E150">
+        <f>COUNTIF('Cook log'!C2:C1000,A150)</f>
+        <v/>
+      </c>
+      <c r="F150" t="n">
+        <v>21</v>
+      </c>
+      <c r="G150">
+        <f>IF(C150="","Never cooked",IF(D150&lt;F150,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Stir-fried baby bok choy</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="C151">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A151)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A151)),"")</f>
+        <v/>
+      </c>
+      <c r="D151">
+        <f>IF(C151="","",TODAY()-C151)</f>
+        <v/>
+      </c>
+      <c r="E151">
+        <f>COUNTIF('Cook log'!C2:C1000,A151)</f>
+        <v/>
+      </c>
+      <c r="F151" t="n">
+        <v>14</v>
+      </c>
+      <c r="G151">
+        <f>IF(C151="","Never cooked",IF(D151&lt;F151,"Cooldown","Due"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update week of 20 Jul: cheese sausage, egg fried rice, ABC soup
- Tue: teriyaki chicken cutlet -> cheese sausage
- Wed: hokkien hai fan -> egg fried rice with char siew
- Thu: dropped steamed egg, added ABC soup (no tomato)
- Synced week file, cook log, and T1 vet

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Teriyaki chicken cutlet</t>
+          <t>Cheese sausage</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Hokkien hai fan (ah gong)</t>
+          <t>Egg fried rice with char siew</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3020,12 +3020,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Steamed egg (ah gong style)</t>
+          <t>ABC soup</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>planned (week of 20 Jul 2026)</t>
+          <t>planned (week of 20 Jul 2026) — no tomato</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8880,6 +8880,68 @@
       </c>
       <c r="G151">
         <f>IF(C151="","Never cooked",IF(D151&lt;F151,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Cheese sausage</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C152">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A152)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A152)),"")</f>
+        <v/>
+      </c>
+      <c r="D152">
+        <f>IF(C152="","",TODAY()-C152)</f>
+        <v/>
+      </c>
+      <c r="E152">
+        <f>COUNTIF('Cook log'!C2:C1000,A152)</f>
+        <v/>
+      </c>
+      <c r="F152" t="n">
+        <v>14</v>
+      </c>
+      <c r="G152">
+        <f>IF(C152="","Never cooked",IF(D152&lt;F152,"Cooldown","Due"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Egg fried rice with char siew</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C153">
+        <f>IFERROR(IF(MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A153)=0,"",MAXIFS('Cook log'!A2:A1000,'Cook log'!C2:C1000,A153)),"")</f>
+        <v/>
+      </c>
+      <c r="D153">
+        <f>IF(C153="","",TODAY()-C153)</f>
+        <v/>
+      </c>
+      <c r="E153">
+        <f>COUNTIF('Cook log'!C2:C1000,A153)</f>
+        <v/>
+      </c>
+      <c r="F153" t="n">
+        <v>21</v>
+      </c>
+      <c r="G153">
+        <f>IF(C153="","Never cooked",IF(D153&lt;F153,"Cooldown","Due"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add week of 28 Sep 2026, oxtail + hey zho recipes, and 21 Sep cook log
Week file for 28 Sep 2026, including the Sunday 27 Sep Cubano extra and the
decisions log (oxtail replacing mei cai kou rou, Hainanese over red-wine
version, beef shank fallback, pulled pork on sliced bread not buns).

Recipes:
- Hainanese oxtail stew (Meatmen Channel) - 2hr tomato/stock braise, serves 4-6
- Red wine braised oxtail (West Country Kitchen) - 4-5hr oven braise, serves 3-4
- Hey zho (prawn rolls) - makes 13 rolls / 39 pieces, steamed then deep-fried

dish-rotation.xlsx:
- Cook log: 15 rows filled in for the week of 21 Sep 2026
- Dish rotation: added Pan-fried salmon (Fish, cd21), Braised oxtail
  (Hainanese style) and Braised oxtail (red wine) (both Beef, cd28)
- Hey zho row annotated with its recipe path and yield

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cook log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dish rotation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cook log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dish rotation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cook log'!$A$1:$D$300</definedName>
@@ -4684,108 +4684,288 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n"/>
+      <c r="A220" s="8" t="n">
+        <v>46285</v>
+      </c>
       <c r="B220" s="3">
         <f>IF(A220="","",TEXT(A220,"ddd"))</f>
         <v/>
       </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>Curry fish head 咖喱鱼头</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>planned Sunday extra (week of 21 Sep 2026) - fish FILLET not head</t>
+        </is>
+      </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n"/>
+      <c r="A221" s="8" t="n">
+        <v>46286</v>
+      </c>
       <c r="B221" s="3">
         <f>IF(A221="","",TEXT(A221,"ddd"))</f>
         <v/>
       </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Chicken parm sandwich</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - served as CUTLETS, no sandwich, half breast each; chilli flakes omitted</t>
+        </is>
+      </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n"/>
+      <c r="A222" s="8" t="n">
+        <v>46286</v>
+      </c>
       <c r="B222" s="3">
         <f>IF(A222="","",TEXT(A222,"ddd"))</f>
         <v/>
       </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Mushroom soup</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n"/>
+      <c r="A223" s="8" t="n">
+        <v>46286</v>
+      </c>
       <c r="B223" s="3">
         <f>IF(A223="","",TEXT(A223,"ddd"))</f>
         <v/>
       </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>Roasted vegetables (oven)</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - basil folded in hot</t>
+        </is>
+      </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n"/>
+      <c r="A224" s="8" t="n">
+        <v>46287</v>
+      </c>
       <c r="B224" s="3">
         <f>IF(A224="","",TEXT(A224,"ddd"))</f>
         <v/>
       </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>Teochew braised duck</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - per week file; Ah Gong version was being developed same week, confirm which was actually cooked</t>
+        </is>
+      </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n"/>
+      <c r="A225" s="8" t="n">
+        <v>46287</v>
+      </c>
       <c r="B225" s="3">
         <f>IF(A225="","",TEXT(A225,"ddd"))</f>
         <v/>
       </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n"/>
+      <c r="A226" s="8" t="n">
+        <v>46288</v>
+      </c>
       <c r="B226" s="3">
         <f>IF(A226="","",TEXT(A226,"ddd"))</f>
         <v/>
       </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>Kong bak pau (braised pork buns)</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - frozen mantou; scaled down from 25 servings</t>
+        </is>
+      </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n"/>
+      <c r="A227" s="8" t="n">
+        <v>46288</v>
+      </c>
       <c r="B227" s="3">
         <f>IF(A227="","",TEXT(A227,"ddd"))</f>
         <v/>
       </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried dou miao</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n"/>
+      <c r="A228" s="8" t="n">
+        <v>46288</v>
+      </c>
       <c r="B228" s="3">
         <f>IF(A228="","",TEXT(A228,"ddd"))</f>
         <v/>
       </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>Hot and sour soup</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n"/>
+      <c r="A229" s="8" t="n">
+        <v>46289</v>
+      </c>
       <c r="B229" s="3">
         <f>IF(A229="","",TEXT(A229,"ddd"))</f>
         <v/>
       </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>Balinese braised beef</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - FIRST COOK</t>
+        </is>
+      </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n"/>
+      <c r="A230" s="8" t="n">
+        <v>46289</v>
+      </c>
       <c r="B230" s="3">
         <f>IF(A230="","",TEXT(A230,"ddd"))</f>
         <v/>
       </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>Hainanese chap chye</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n"/>
+      <c r="A231" s="8" t="n">
+        <v>46289</v>
+      </c>
       <c r="B231" s="3">
         <f>IF(A231="","",TEXT(A231,"ddd"))</f>
         <v/>
       </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>Chinese yam and chicken soup</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - PORK RIB version; EARLY 16d after 8 Sep, cd 21; user approved</t>
+        </is>
+      </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n"/>
+      <c r="A232" s="8" t="n">
+        <v>46290</v>
+      </c>
       <c r="B232" s="3">
         <f>IF(A232="","",TEXT(A232,"ddd"))</f>
         <v/>
       </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>Taiwanese fried rice</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n"/>
+      <c r="A233" s="8" t="n">
+        <v>46290</v>
+      </c>
       <c r="B233" s="3">
         <f>IF(A233="","",TEXT(A233,"ddd"))</f>
         <v/>
       </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>Wasabi mayo prawns</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - Kewpie mayo instead of from-scratch</t>
+        </is>
+      </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n"/>
+      <c r="A234" s="8" t="n">
+        <v>46290</v>
+      </c>
       <c r="B234" s="3">
         <f>IF(A234="","",TEXT(A234,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>Radish pork rib soup with dates</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 21 Sep 2026) - EARLY 14d after 11 Sep, cd 21; user approved</t>
+        </is>
       </c>
     </row>
     <row r="235">
@@ -5267,7 +5447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7090,7 +7270,11 @@
         <f>IF(C57="","Never cooked",IF(D57&lt;F57,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H57" s="4" t="inlineStr"/>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>recipes/hey-zho.md - makes 13 rolls / 39 pieces; steamed 15 min, cooled, cornflour-coated, deep-fried. Needs 1kg peeled prawns, 5-spice beancurd skin. Never cooked</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -10949,6 +11133,66 @@
       <c r="H186" s="3" t="inlineStr">
         <is>
           <t>recipes/braised-duck-ah-gong-recipe.md - Fully confirmed via Ah Gong's own WhatsApp messages. Separate rotation entry so it doesn't collide with the Teochew version. Never cooked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>Pan-fried salmon</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>Fish</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="H187" s="3" t="inlineStr">
+        <is>
+          <t>Household - no recipe file; added 24 Sep. Fully cook through</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>Braised oxtail (Hainanese style)</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>Beef</t>
+        </is>
+      </c>
+      <c r="F188" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H188" s="3" t="inlineStr">
+        <is>
+          <t>recipes/hainanese-oxtail-stew.md - Meatmen Channel; 2hr braise, oxtail floured+fried first. Serves 4-6 on 2kg. Never cooked</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>Braised oxtail (red wine)</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>Beef</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H189" s="3" t="inlineStr">
+        <is>
+          <t>recipes/red-wine-braised-oxtail.md - West Country Kitchen; oven braise 4-5hr at 140-150C, served on mash. Serves 3-4, oxtail weight not stated. Never cooked</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish week of 5 Oct 2026: vet, market list, cook log; helper is now Jayzel
- Add pregnancy vet and final market list for the week of 5 Oct
- Swap Tuesday's Thai fish cakes for fried chicken wings
- Pre-scale japchae and yam pork belly to 5.5 pax; complete the Thai fish cake recipe
- Log the week in the cook log; add 13 new inventory items
- Rename the helper from Mia to Jayzel in both skills

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -5273,94 +5273,250 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="2" t="n"/>
+      <c r="A251" s="8" t="n">
+        <v>46299</v>
+      </c>
       <c r="B251" s="3">
         <f>IF(A251="","",TEXT(A251,"ddd"))</f>
         <v/>
       </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>Japchae 잡채</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>planned Sunday extra (week of 5 Oct 2026) - FIRST COOK; recipes/japchae.md pre-scaled 5.5</t>
+        </is>
+      </c>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="n"/>
+      <c r="A252" s="8" t="n">
+        <v>46300</v>
+      </c>
       <c r="B252" s="3">
         <f>IF(A252="","",TEXT(A252,"ddd"))</f>
         <v/>
       </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>Hakka yam pork belly 芋头扣肉</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - FIRST COOK; steam Sun night, rice cooker busy Mon</t>
+        </is>
+      </c>
     </row>
     <row r="253">
-      <c r="A253" s="2" t="n"/>
+      <c r="A253" s="8" t="n">
+        <v>46300</v>
+      </c>
       <c r="B253" s="3">
         <f>IF(A253="","",TEXT(A253,"ddd"))</f>
         <v/>
       </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Stir-fried eggs with Chinese sausage 腊肠炒蛋</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - FIRST COOK; household, no recipe; eggs cooked firm</t>
+        </is>
+      </c>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="n"/>
+      <c r="A254" s="8" t="n">
+        <v>46300</v>
+      </c>
       <c r="B254" s="3">
         <f>IF(A254="","",TEXT(A254,"ddd"))</f>
         <v/>
       </c>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>Watercress pork rib soup</t>
+        </is>
+      </c>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - picked by Claude - Monday soup was "no bamboo shoot"</t>
+        </is>
+      </c>
     </row>
     <row r="255">
-      <c r="A255" s="2" t="n"/>
+      <c r="A255" s="8" t="n">
+        <v>46300</v>
+      </c>
       <c r="B255" s="3">
         <f>IF(A255="","",TEXT(A255,"ddd"))</f>
         <v/>
       </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="n"/>
+      <c r="A256" s="8" t="n">
+        <v>46301</v>
+      </c>
       <c r="B256" s="3">
         <f>IF(A256="","",TEXT(A256,"ddd"))</f>
         <v/>
       </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>Steamed baby threadfin</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - picked by Claude for "some steamed fish"</t>
+        </is>
+      </c>
     </row>
     <row r="257">
-      <c r="A257" s="2" t="n"/>
+      <c r="A257" s="8" t="n">
+        <v>46301</v>
+      </c>
       <c r="B257" s="3">
         <f>IF(A257="","",TEXT(A257,"ddd"))</f>
         <v/>
       </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>Fried chicken wings</t>
+        </is>
+      </c>
+      <c r="D257" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - replaced Thai fishcakes (user, 3 Oct); ~1.6kg wings</t>
+        </is>
+      </c>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="n"/>
+      <c r="A258" s="8" t="n">
+        <v>46301</v>
+      </c>
       <c r="B258" s="3">
         <f>IF(A258="","",TEXT(A258,"ddd"))</f>
         <v/>
       </c>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="259">
-      <c r="A259" s="2" t="n"/>
+      <c r="A259" s="8" t="n">
+        <v>46301</v>
+      </c>
       <c r="B259" s="3">
         <f>IF(A259="","",TEXT(A259,"ddd"))</f>
         <v/>
       </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="260">
-      <c r="A260" s="2" t="n"/>
+      <c r="A260" s="8" t="n">
+        <v>46302</v>
+      </c>
       <c r="B260" s="3">
         <f>IF(A260="","",TEXT(A260,"ddd"))</f>
         <v/>
       </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>Japanese curry rice</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - ~600g chicken (estimate); chilli reduced for the child</t>
+        </is>
+      </c>
     </row>
     <row r="261">
-      <c r="A261" s="2" t="n"/>
+      <c r="A261" s="8" t="n">
+        <v>46302</v>
+      </c>
       <c r="B261" s="3">
         <f>IF(A261="","",TEXT(A261,"ddd"))</f>
         <v/>
       </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>Fishball soup with cabbage</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - FIRST COOK; picked by Claude; household, no recipe</t>
+        </is>
+      </c>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="n"/>
+      <c r="A262" s="8" t="n">
+        <v>46304</v>
+      </c>
       <c r="B262" s="3">
         <f>IF(A262="","",TEXT(A262,"ddd"))</f>
         <v/>
       </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>Shepherd's pie</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - lamb ~1kg for 5.5 (or beef)</t>
+        </is>
+      </c>
     </row>
     <row r="263">
-      <c r="A263" s="2" t="n"/>
+      <c r="A263" s="8" t="n">
+        <v>46304</v>
+      </c>
       <c r="B263" s="3">
         <f>IF(A263="","",TEXT(A263,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>Mushroom soup</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 5 Oct 2026) - EARLY 18d after 21 Sep, cd 28; user approved; no cream this time</t>
+        </is>
       </c>
     </row>
     <row r="264">
@@ -7500,7 +7656,7 @@
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>recipes/thai-fish-cakes.md - restored 3 Oct from git (Tod Mun Pla); ingredient list only, NO quantities yet</t>
+          <t>recipes/thai-fish-cakes.md - PRE-SCALED to 5.5 pax (x1.6); original video ingredients + user-supplied guide quantities. Deep-fried; spicy (red curry paste)</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11232,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Household - Mia improvises</t>
+          <t>Household - no recipe file. Was Mia's dish; Mia briefed Jayzel on household dishes before leaving 3 Oct 2026 - check Jayzel knows this one</t>
         </is>
       </c>
     </row>
@@ -11148,7 +11304,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Household - Mia knows it</t>
+          <t>Household - no recipe file. Was Mia's dish; Mia briefed Jayzel on household dishes before leaving 3 Oct 2026 - check Jayzel knows this one</t>
         </is>
       </c>
     </row>
@@ -11404,7 +11560,7 @@
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>recipes/hakka-yam-pork-belly.md - serves 6-8; marinate 1hr, pan-fry, steam 1.5hr in a rice cooker. Never cooked</t>
+          <t>recipes/hakka-yam-pork-belly.md - PRE-SCALED to 5.5 pax (x0.8 from source 6-8); marinate 1hr, pan-fry, steam 1.5hr. Never cooked</t>
         </is>
       </c>
     </row>
@@ -11444,7 +11600,7 @@
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>recipes/japchae.md - serves 3-4 as written (100g noodles, 50g beef). Never cooked</t>
+          <t>recipes/japchae.md - PRE-SCALED to 5.5 pax (x1.6 from source 3-4). Side-dish portions: 80g beef. Never cooked</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add weeks of 12 and 19 Oct 2026, with step-by-step cooking instructions
- Week of 12 Oct: menu (5 pax), pregnancy vet, the user's final market list,
  cook log and inventory; black pepper beef recipe from the user's paste
- Week of 19 Oct: menu, vet, confirmed market list with gaps, and the new
  step-by-step instructions, one WhatsApp message per day
- New recipe: steamed fish paste with minced pork (the family's own)
- Household versions added to the green curry, glutinous rice, Thai seabass,
  si ji dou sambal, yam rice, wings, fishball soup and pad kra pao recipes
- weekly-menu skill: now 12 steps (market list confirmation, step-by-step
  instructions), Sunday for 3, portion, chilli and bean-prep rules
- Cook log, rotation rows and inventory updated for both weeks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dish-rotation.xlsx
+++ b/dish-rotation.xlsx
@@ -5520,227 +5520,611 @@
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="n"/>
+      <c r="A264" s="8" t="n">
+        <v>46306</v>
+      </c>
       <c r="B264" s="3">
         <f>IF(A264="","",TEXT(A264,"ddd"))</f>
         <v/>
       </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>Beef hayashi rice</t>
+        </is>
+      </c>
+      <c r="D264" s="3" t="inlineStr">
+        <is>
+          <t>planned Sunday extra (week of 12 Oct 2026) - FIRST COOK; as written</t>
+        </is>
+      </c>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="n"/>
+      <c r="A265" s="8" t="n">
+        <v>46307</v>
+      </c>
       <c r="B265" s="3">
         <f>IF(A265="","",TEXT(A265,"ddd"))</f>
         <v/>
       </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>Greek lemon chicken</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - FIRST COOK; the 5 thighs at home; marinade x0.6</t>
+        </is>
+      </c>
     </row>
     <row r="266">
-      <c r="A266" s="2" t="n"/>
+      <c r="A266" s="8" t="n">
+        <v>46307</v>
+      </c>
       <c r="B266" s="3">
         <f>IF(A266="","",TEXT(A266,"ddd"))</f>
         <v/>
       </c>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>Crispy roast potatoes</t>
+        </is>
+      </c>
+      <c r="D266" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - recipes/roast-potatoes.md 1.5kg</t>
+        </is>
+      </c>
     </row>
     <row r="267">
-      <c r="A267" s="2" t="n"/>
+      <c r="A267" s="8" t="n">
+        <v>46307</v>
+      </c>
       <c r="B267" s="3">
         <f>IF(A267="","",TEXT(A267,"ddd"))</f>
         <v/>
       </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>Roasted vegetables (oven)</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - no potato wedges; x1.25</t>
+        </is>
+      </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="n"/>
+      <c r="A268" s="8" t="n">
+        <v>46308</v>
+      </c>
       <c r="B268" s="3">
         <f>IF(A268="","",TEXT(A268,"ddd"))</f>
         <v/>
       </c>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>Steamed pomfret</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - 2 fish 500-600g, steamed one at a time</t>
+        </is>
+      </c>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="n"/>
+      <c r="A269" s="8" t="n">
+        <v>46308</v>
+      </c>
       <c r="B269" s="3">
         <f>IF(A269="","",TEXT(A269,"ddd"))</f>
         <v/>
       </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried dou miao</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - x2</t>
+        </is>
+      </c>
     </row>
     <row r="270">
-      <c r="A270" s="2" t="n"/>
+      <c r="A270" s="8" t="n">
+        <v>46308</v>
+      </c>
       <c r="B270" s="3">
         <f>IF(A270="","",TEXT(A270,"ddd"))</f>
         <v/>
       </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>Pork rib king</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - x1.5; method in the video</t>
+        </is>
+      </c>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="n"/>
+      <c r="A271" s="8" t="n">
+        <v>46309</v>
+      </c>
       <c r="B271" s="3">
         <f>IF(A271="","",TEXT(A271,"ddd"))</f>
         <v/>
       </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>Chicken curry</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - dried chillies cut to 3-4</t>
+        </is>
+      </c>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="n"/>
+      <c r="A272" s="8" t="n">
+        <v>46309</v>
+      </c>
       <c r="B272" s="3">
         <f>IF(A272="","",TEXT(A272,"ddd"))</f>
         <v/>
       </c>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>Frozen prata</t>
+        </is>
+      </c>
+      <c r="D272" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - store-bought</t>
+        </is>
+      </c>
     </row>
     <row r="273">
-      <c r="A273" s="2" t="n"/>
+      <c r="A273" s="8" t="n">
+        <v>46310</v>
+      </c>
       <c r="B273" s="3">
         <f>IF(A273="","",TEXT(A273,"ddd"))</f>
         <v/>
       </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>Black pepper beef</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - FIRST COOK; 400g; method inferred</t>
+        </is>
+      </c>
     </row>
     <row r="274">
-      <c r="A274" s="2" t="n"/>
+      <c r="A274" s="8" t="n">
+        <v>46310</v>
+      </c>
       <c r="B274" s="3">
         <f>IF(A274="","",TEXT(A274,"ddd"))</f>
         <v/>
       </c>
+      <c r="C274" s="3" t="inlineStr">
+        <is>
+          <t>Water steamed egg</t>
+        </is>
+      </c>
+      <c r="D274" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - FIRST COOK; no meat; set through</t>
+        </is>
+      </c>
     </row>
     <row r="275">
-      <c r="A275" s="2" t="n"/>
+      <c r="A275" s="8" t="n">
+        <v>46310</v>
+      </c>
       <c r="B275" s="3">
         <f>IF(A275="","",TEXT(A275,"ddd"))</f>
         <v/>
       </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried French beans with dried shrimp</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - FIRST COOK; as written</t>
+        </is>
+      </c>
     </row>
     <row r="276">
-      <c r="A276" s="2" t="n"/>
+      <c r="A276" s="8" t="n">
+        <v>46311</v>
+      </c>
       <c r="B276" s="3">
         <f>IF(A276="","",TEXT(A276,"ddd"))</f>
         <v/>
       </c>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>Taiwanese braised pork rice</t>
+        </is>
+      </c>
+      <c r="D276" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 12 Oct 2026) - as written; method in the video</t>
+        </is>
+      </c>
     </row>
     <row r="277">
-      <c r="A277" s="2" t="n"/>
+      <c r="A277" s="8" t="n">
+        <v>46313</v>
+      </c>
       <c r="B277" s="3">
         <f>IF(A277="","",TEXT(A277,"ddd"))</f>
         <v/>
       </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>Green curry</t>
+        </is>
+      </c>
+      <c r="D277" s="3" t="inlineStr">
+        <is>
+          <t>planned Sunday extra (week of 19 Oct 2026) - FIRST COOK; Sunday extra for 3; Dancing Chef packet; eggplant, long beans, carrot</t>
+        </is>
+      </c>
     </row>
     <row r="278">
-      <c r="A278" s="2" t="n"/>
+      <c r="A278" s="8" t="n">
+        <v>46313</v>
+      </c>
       <c r="B278" s="3">
         <f>IF(A278="","",TEXT(A278,"ddd"))</f>
         <v/>
       </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>planned Sunday extra (week of 19 Oct 2026) - jasmine rice, 3 cups (for 3 pax)</t>
+        </is>
+      </c>
     </row>
     <row r="279">
-      <c r="A279" s="2" t="n"/>
+      <c r="A279" s="8" t="n">
+        <v>46314</v>
+      </c>
       <c r="B279" s="3">
         <f>IF(A279="","",TEXT(A279,"ddd"))</f>
         <v/>
       </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Fragrant glutinous rice</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - FIRST COOK; for 5.5 pax; + 300g pork belly; wok then rice cooker, water 1:1; soak 2h</t>
+        </is>
+      </c>
     </row>
     <row r="280">
-      <c r="A280" s="2" t="n"/>
+      <c r="A280" s="8" t="n">
+        <v>46314</v>
+      </c>
       <c r="B280" s="3">
         <f>IF(A280="","",TEXT(A280,"ddd"))</f>
         <v/>
       </c>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - choy sum</t>
+        </is>
+      </c>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="n"/>
+      <c r="A281" s="8" t="n">
+        <v>46315</v>
+      </c>
       <c r="B281" s="3">
         <f>IF(A281="","",TEXT(A281,"ddd"))</f>
         <v/>
       </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>Thai style steamed seabass</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - one fish; sauce finely chopped and simmered; chilli seeds out; no cabbage</t>
+        </is>
+      </c>
     </row>
     <row r="282">
-      <c r="A282" s="2" t="n"/>
+      <c r="A282" s="8" t="n">
+        <v>46315</v>
+      </c>
       <c r="B282" s="3">
         <f>IF(A282="","",TEXT(A282,"ddd"))</f>
         <v/>
       </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried French beans with dried shrimp</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - EARLY 5d after 15 Oct, cd 21; user approved; si ji dou; user asked for it again; now with a dried shrimp sambal (NoobCook technique)</t>
+        </is>
+      </c>
     </row>
     <row r="283">
-      <c r="A283" s="2" t="n"/>
+      <c r="A283" s="8" t="n">
+        <v>46315</v>
+      </c>
       <c r="B283" s="3">
         <f>IF(A283="","",TEXT(A283,"ddd"))</f>
         <v/>
       </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>Steamed fish paste with minced meat</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - FIRST COOK; user's recipe, garlic-heavy, steam 15 min</t>
+        </is>
+      </c>
     </row>
     <row r="284">
-      <c r="A284" s="2" t="n"/>
+      <c r="A284" s="8" t="n">
+        <v>46315</v>
+      </c>
       <c r="B284" s="3">
         <f>IF(A284="","",TEXT(A284,"ddd"))</f>
         <v/>
       </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="285">
-      <c r="A285" s="2" t="n"/>
+      <c r="A285" s="8" t="n">
+        <v>46316</v>
+      </c>
       <c r="B285" s="3">
         <f>IF(A285="","",TEXT(A285,"ddd"))</f>
         <v/>
       </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>Yam rice</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - FIRST COOK; with pork belly</t>
+        </is>
+      </c>
     </row>
     <row r="286">
-      <c r="A286" s="2" t="n"/>
+      <c r="A286" s="8" t="n">
+        <v>46316</v>
+      </c>
       <c r="B286" s="3">
         <f>IF(A286="","",TEXT(A286,"ddd"))</f>
         <v/>
       </c>
+      <c r="C286" s="3" t="inlineStr">
+        <is>
+          <t>Baked chicken wings</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - FIRST COOK; 12 individually frozen mid wings (2 per person)</t>
+        </is>
+      </c>
     </row>
     <row r="287">
-      <c r="A287" s="2" t="n"/>
+      <c r="A287" s="8" t="n">
+        <v>46316</v>
+      </c>
       <c r="B287" s="3">
         <f>IF(A287="","",TEXT(A287,"ddd"))</f>
         <v/>
       </c>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>Fishball soup with cabbage</t>
+        </is>
+      </c>
+      <c r="D287" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - EARLY 14d after 7 Oct, cd 21; user approved; fishballs and wawa vegetable, no pork (user, 18 Oct)</t>
+        </is>
+      </c>
     </row>
     <row r="288">
-      <c r="A288" s="2" t="n"/>
+      <c r="A288" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="B288" s="3">
         <f>IF(A288="","",TEXT(A288,"ddd"))</f>
         <v/>
       </c>
+      <c r="C288" s="3" t="inlineStr">
+        <is>
+          <t>Pan-fried threadfin with leek</t>
+        </is>
+      </c>
+      <c r="D288" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - household</t>
+        </is>
+      </c>
     </row>
     <row r="289">
-      <c r="A289" s="2" t="n"/>
+      <c r="A289" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="B289" s="3">
         <f>IF(A289="","",TEXT(A289,"ddd"))</f>
         <v/>
       </c>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>Enoki with pork wrap</t>
+        </is>
+      </c>
+      <c r="D289" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - FIRST COOK; 16 rolls; enoki cooked soft</t>
+        </is>
+      </c>
     </row>
     <row r="290">
-      <c r="A290" s="2" t="n"/>
+      <c r="A290" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="B290" s="3">
         <f>IF(A290="","",TEXT(A290,"ddd"))</f>
         <v/>
       </c>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="291">
-      <c r="A291" s="2" t="n"/>
+      <c r="A291" s="8" t="n">
+        <v>46317</v>
+      </c>
       <c r="B291" s="3">
         <f>IF(A291="","",TEXT(A291,"ddd"))</f>
         <v/>
       </c>
+      <c r="C291" s="3" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="D291" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - my addition</t>
+        </is>
+      </c>
     </row>
     <row r="292">
-      <c r="A292" s="2" t="n"/>
+      <c r="A292" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="B292" s="3">
         <f>IF(A292="","",TEXT(A292,"ddd"))</f>
         <v/>
       </c>
+      <c r="C292" s="3" t="inlineStr">
+        <is>
+          <t>Pork krapow (Pad Kra Pao)</t>
+        </is>
+      </c>
+      <c r="D292" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - 500g pork; chilli seeds out; yolk firm; no prik nam pla</t>
+        </is>
+      </c>
     </row>
     <row r="293">
-      <c r="A293" s="2" t="n"/>
+      <c r="A293" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="B293" s="3">
         <f>IF(A293="","",TEXT(A293,"ddd"))</f>
         <v/>
       </c>
+      <c r="C293" s="3" t="inlineStr">
+        <is>
+          <t>Stir-fried eggs and prawns</t>
+        </is>
+      </c>
+      <c r="D293" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026) - household</t>
+        </is>
+      </c>
     </row>
     <row r="294">
-      <c r="A294" s="2" t="n"/>
+      <c r="A294" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="B294" s="3">
         <f>IF(A294="","",TEXT(A294,"ddd"))</f>
         <v/>
       </c>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried vegetable</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="n"/>
+      <c r="A295" s="8" t="n">
+        <v>46318</v>
+      </c>
       <c r="B295" s="3">
         <f>IF(A295="","",TEXT(A295,"ddd"))</f>
         <v/>
+      </c>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>Steamed rice</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="inlineStr">
+        <is>
+          <t>planned (week of 19 Oct 2026)</t>
+        </is>
       </c>
     </row>
     <row r="296">
@@ -5795,7 +6179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5976,7 +6360,11 @@
         <f>IF(C5="","Never cooked",IF(D5&lt;F5,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>recipes/pork-rib-king.md - ingredients only, method in the video (0WXGuOQq_xU). x1.5 for 5 pax</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -6264,7 +6652,11 @@
         <f>IF(C14="","Never cooked",IF(D14&lt;F14,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>recipes/roasted-vegetables.md - ingredients only; x1.25 for 5 pax; potato wedges left out when roast potatoes are served</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -6328,7 +6720,11 @@
         <f>IF(C16="","Never cooked",IF(D16&lt;F16,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>recipes/taiwanese-braised-pork-rice.md - ingredients only, method in the video (hqcVtqGoRG0)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -6360,7 +6756,11 @@
         <f>IF(C17="","Never cooked",IF(D17&lt;F17,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>recipes/steamed-fish-paste-with-minced-pork.md - user's own recipe, revised 17 Oct 2026: pork 1/3 and garlic paste 1/4-1/3 of the fish paste by volume; oil on top; steam 15 min. Never cooked</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -6584,7 +6984,11 @@
         <f>IF(C24="","Never cooked",IF(D24&lt;F24,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H24" s="4" t="inlineStr"/>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>recipes/soy-and-oyster-sauce-wings.md - oven method; individually frozen mid wings, x0.6 marinade. Never cooked</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -6744,7 +7148,11 @@
         <f>IF(C29="","Never cooked",IF(D29&lt;F29,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>recipes/thai-style-steamed-fish.md - ingredients only, method in the video (-2hNdMmJogU); one 700g fish, chillies cut to 4-5</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -6904,7 +7312,11 @@
         <f>IF(C34="","Never cooked",IF(D34&lt;F34,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H34" s="4" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>recipes/yam-rice.md - pork belly version (user, 17 Oct 2026), x1.6. Never cooked</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -7786,7 +8198,11 @@
         <f>IF(C62="","Never cooked",IF(D62&lt;F62,"Cooldown","Due"))</f>
         <v/>
       </c>
-      <c r="H62" s="4" t="inlineStr"/>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>recipes/thai-green-curry.md - Dancing Chef packet; eggplant, long beans, carrot (the user's usual); Sunday for 3 pax</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -8855,6 +9271,11 @@
         <f>IF(C101="","Never cooked",IF(D101&lt;F101,"Cooldown","Due"))</f>
         <v/>
       </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Household - no recipe file. Eggs cooked firm, prawns opaque</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -9692,6 +10113,11 @@
         <f>IF(C128="","Never cooked",IF(D128&lt;F128,"Cooldown","Due"))</f>
         <v/>
       </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>recipes/roast-potatoes.md - 1.5kg for 5 pax; skip the raw parsley</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -10188,6 +10614,11 @@
         <f>IF(C144="","Never cooked",IF(D144&lt;F144,"Cooldown","Due"))</f>
         <v/>
       </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>recipes/chicken-curry-potato.md - 4-6 pax as written; cut dried chillies to 3-4 for the child</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -11601,6 +12032,146 @@
       <c r="H192" s="3" t="inlineStr">
         <is>
           <t>recipes/japchae.md - PRE-SCALED to 5.5 pax (x1.6 from source 3-4). Side-dish portions: 80g beef. Never cooked</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t>Beef hayashi rice</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>Beef</t>
+        </is>
+      </c>
+      <c r="F193" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H193" s="3" t="inlineStr">
+        <is>
+          <t>recipes/hayashi-rice.md - 2h simmer, as written (~5-6 pax). Never cooked. Added 9 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>Greek lemon chicken</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="H194" s="3" t="inlineStr">
+        <is>
+          <t>recipes/greek-lemon-chicken.md - written for 8 bone-in thighs; made with 5 (marinade x0.6); own lemon rice and green beans not made. Never cooked</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>Black pepper beef</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>Beef</t>
+        </is>
+      </c>
+      <c r="F195" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="H195" s="3" t="inlineStr">
+        <is>
+          <t>recipes/black-pepper-beef.md - method inferred; 400g for 5 pax. Never cooked</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>Water steamed egg</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>Egg</t>
+        </is>
+      </c>
+      <c r="F196" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="H196" s="3" t="inlineStr">
+        <is>
+          <t>Plain, no meat. Ah Gong steamed egg mix (recipes/steamed-egg.md) without the pork; 5 eggs for 5 pax; steam until set</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>Stir fried French beans with dried shrimp</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>Vegetable</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="H197" s="3" t="inlineStr">
+        <is>
+          <t>recipes/zi-char-french-beans-with-dried-shrimp.md - as written (500g). Never cooked</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>Fragrant glutinous rice</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="F198" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="H198" s="3" t="inlineStr">
+        <is>
+          <t>recipes/fragrant-glutinous-rice.md - household version (18 Oct 2026): + 300g pork belly, 2 sausages, wok then ordinary rice cooker, water 1:1, steam longer; soak 2h. Never cooked</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>Enoki with pork wrap</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="H199" s="3" t="inlineStr">
+        <is>
+          <t>recipes/enoki-mushroom-meat-roll.md - made with pork shabu slices, x2 (16 rolls). Enoki must be cooked soft and hot. Never cooked</t>
         </is>
       </c>
     </row>

</xml_diff>